<commit_message>
INTERIM edits for soft cap and reliability redesign
</commit_message>
<xml_diff>
--- a/InputData/elec/HCFoTC/Hard Cap Frac of Total Capacity.xlsx
+++ b/InputData/elec/HCFoTC/Hard Cap Frac of Total Capacity.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\elec\HCFoTC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us-dev-sandbox\InputData\elec\HCFoTC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E8D0CE3-CBFC-4D0A-8776-52CEC165498F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEAD68AA-083D-4300-9600-878FDA94FC37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{D718C537-5235-45E1-A117-07B097D2BDF0}"/>
+    <workbookView xWindow="-23820" yWindow="3465" windowWidth="21600" windowHeight="12645" activeTab="1" xr2:uid="{D718C537-5235-45E1-A117-07B097D2BDF0}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -264,11 +264,10 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma 2" xfId="5" xr:uid="{68733429-A9FA-4187-B93D-3BEA15728D17}"/>
@@ -754,7 +753,7 @@
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+      <c r="A7" t="s">
         <v>7</v>
       </c>
     </row>
@@ -788,7 +787,7 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>